<commit_message>
Fix: Strict tab role separation and removed test user
</commit_message>
<xml_diff>
--- a/Live_Setup/Quote_Bank_Resources_Manager/categories.xlsx
+++ b/Live_Setup/Quote_Bank_Resources_Manager/categories.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Quote_Bank_Resources_Manager\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\RONE_Studio\RONE_MentorOS\Live_Setup\Quote_Bank_Resources_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0223AE4E-91D1-46B1-8A65-3E2F8469EA23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0574C197-B983-45F7-AFF7-188EA5DE465F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
   <si>
     <t>Category</t>
   </si>
@@ -77,97 +77,106 @@
     <t>GS Paper 1</t>
   </si>
   <si>
-    <t>rank 1 shruti sharma</t>
-  </si>
-  <si>
-    <t>rank 111 kashish kalra</t>
-  </si>
-  <si>
-    <t>rank 156 zinnia aurora</t>
-  </si>
-  <si>
-    <t>rank 210 sania seervi</t>
-  </si>
-  <si>
-    <t>rank 37 shobhika pathak</t>
-  </si>
-  <si>
-    <t>rank 50 k n chandana jahnavi</t>
-  </si>
-  <si>
-    <t>rank 9 nausheen</t>
-  </si>
-  <si>
-    <t>rank 289 chandar prabha sharma</t>
-  </si>
-  <si>
-    <t>rank 399 oishee mandal</t>
-  </si>
-  <si>
-    <t>rank 100 vijeta b hosamani</t>
-  </si>
-  <si>
-    <t>rank 127 aditi upadhyay</t>
-  </si>
-  <si>
-    <t>rank 189 poorva agrawal</t>
-  </si>
-  <si>
-    <t>rank 194 aditi yadav</t>
-  </si>
-  <si>
-    <t>rank 199 tripti kalhans</t>
-  </si>
-  <si>
-    <t>rank 204 shubhra panda</t>
-  </si>
-  <si>
-    <t>rank 99 annapurna singh</t>
-  </si>
-  <si>
-    <t>rank 25 ritika verma</t>
-  </si>
-  <si>
-    <t>rank 26 rupal rana</t>
-  </si>
-  <si>
-    <t>rank 36 ayushi pradhan</t>
-  </si>
-  <si>
-    <t>rank 39 deepti rohilla</t>
-  </si>
-  <si>
-    <t>rank 51 rajput neha uddhavsingh</t>
-  </si>
-  <si>
-    <t>rank 17 swati sharma</t>
-  </si>
-  <si>
-    <t>rank 61 khushhali solanki</t>
-  </si>
-  <si>
-    <t>rank 65 chhaya singh</t>
-  </si>
-  <si>
-    <t>rank 80 garima mundra</t>
-  </si>
-  <si>
-    <t>rank 18 wardah khan</t>
-  </si>
-  <si>
-    <t>rank 263 girisha chaudhary</t>
-  </si>
-  <si>
-    <t>rank 1 shakti dubey</t>
-  </si>
-  <si>
-    <t>rank 189 anupriya rai</t>
-  </si>
-  <si>
-    <t>rank 40 iram choudhary</t>
-  </si>
-  <si>
-    <t>rank 7 aayushi bansal</t>
+    <t>RANK 1 SHRUTI SHARMA</t>
+  </si>
+  <si>
+    <t>RANK 111 KASHISH KALRA</t>
+  </si>
+  <si>
+    <t>RANK 156 ZINNIA AURORA</t>
+  </si>
+  <si>
+    <t>RANK 210 SANIA SEERVI</t>
+  </si>
+  <si>
+    <t>RANK 37 SHOBHIKA PATHAK</t>
+  </si>
+  <si>
+    <t>RANK 50 K N CHANDANA JAHNAVI</t>
+  </si>
+  <si>
+    <t>RANK 9 NAUSHEEN</t>
+  </si>
+  <si>
+    <t>RANK 289 CHANDAR PRABHA SHARMA</t>
+  </si>
+  <si>
+    <t>RANK 399 OISHEE MANDAL</t>
+  </si>
+  <si>
+    <t>RANK 100 VIJETA B HOSAMANI</t>
+  </si>
+  <si>
+    <t>RANK 127 ADITI UPADHYAY</t>
+  </si>
+  <si>
+    <t>RANK 189 POORVA AGRAWAL</t>
+  </si>
+  <si>
+    <t>RANK 194 ADITI YADAV</t>
+  </si>
+  <si>
+    <t>RANK 199 TRIPTI KALHANS</t>
+  </si>
+  <si>
+    <t>RANK 204 SHUBHRA PANDA</t>
+  </si>
+  <si>
+    <t>RANK 99 ANNAPURNA SINGH</t>
+  </si>
+  <si>
+    <t>RANK 25 RITIKA VERMA</t>
+  </si>
+  <si>
+    <t>RANK 26 RUPAL RANA</t>
+  </si>
+  <si>
+    <t>RANK 36 AYUSHI PRADHAN</t>
+  </si>
+  <si>
+    <t>RANK 39 DEEPTI ROHILLA</t>
+  </si>
+  <si>
+    <t>RANK 51 RAJPUT NEHA UDDHAVSINGH</t>
+  </si>
+  <si>
+    <t>RANK 17 SWATI SHARMA</t>
+  </si>
+  <si>
+    <t>RANK 61 KHUSHHALI SOLANKI</t>
+  </si>
+  <si>
+    <t>RANK 65 CHHAYA SINGH</t>
+  </si>
+  <si>
+    <t>RANK 80 GARIMA MUNDRA</t>
+  </si>
+  <si>
+    <t>RANK 18 WARDAH KHAN</t>
+  </si>
+  <si>
+    <t>RANK 263 GIRISHA CHAUDHARY</t>
+  </si>
+  <si>
+    <t>RANK 1 SHAKTI DUBEY</t>
+  </si>
+  <si>
+    <t>RANK 189 ANUPRIYA RAI</t>
+  </si>
+  <si>
+    <t>RANK 40 IRAM CHOUDHARY</t>
+  </si>
+  <si>
+    <t>RANK 7 AAYUSHI BANSAL</t>
+  </si>
+  <si>
+    <t>Quotes Bank</t>
+  </si>
+  <si>
+    <t>All them</t>
+  </si>
+  <si>
+    <t>Your Choice</t>
   </si>
 </sst>
 </file>
@@ -234,7 +243,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -249,6 +268,36 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -548,86 +597,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.5703125" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
     </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -647,205 +693,216 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="1">
-        <v>2021</v>
+      <c r="A2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="1">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="1">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2026</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="21.75" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
+    <row r="23" spans="1:1" ht="21.75" x14ac:dyDescent="0.35">
+      <c r="A23" s="3" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.35">
-      <c r="C33"/>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C34"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1 A34:A1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  <conditionalFormatting sqref="A34:A1048576 A1:A2">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1 A33:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="A35:A1048576 A1:A2">
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>